<commit_message>
#6 U1 part no change into VIPER319XDTR.
</commit_message>
<xml_diff>
--- a/Design-Files/BOM/Smart-Switch-v1.1.xlsx
+++ b/Design-Files/BOM/Smart-Switch-v1.1.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\adamkop-smartswitch\Design-Files\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\adamkop-smartswitch\Design-Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFCA1A3E-F672-4306-9375-B7BD6AAF0304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3552" yWindow="3276" windowWidth="17280" windowHeight="8964" xr2:uid="{45B62AA9-203E-4F71-9C89-11ACADAE83D7}"/>
+    <workbookView xWindow="3555" yWindow="3270" windowWidth="17280" windowHeight="8970"/>
   </bookViews>
   <sheets>
     <sheet name="Smart-Switch-v1.1" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Smart-Switch-v1.1'!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -602,12 +601,6 @@
     <t>SW1, SW2</t>
   </si>
   <si>
-    <t>VIPER319LDTR</t>
-  </si>
-  <si>
-    <t>AC to DC Switching Converter Boost/Buck/Flyback 4.25V 145kHz T/R 16-Pin SO N</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -663,12 +656,18 @@
   </si>
   <si>
     <t>X322540MPB4SI</t>
+  </si>
+  <si>
+    <t>VIPER319XDTR</t>
+  </si>
+  <si>
+    <t>IC OFFLINE SWITCH MULT TOP 16SO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1038,16 +1037,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B661AD3-D2A9-48A4-8456-3F57203F86D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="28.109375" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1067,7 +1066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1087,7 +1086,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1107,7 +1106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
@@ -1127,7 +1126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1147,7 +1146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -1167,7 +1166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
@@ -1187,7 +1186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
@@ -1207,7 +1206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -1227,7 +1226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -1247,7 +1246,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>37</v>
       </c>
@@ -1267,7 +1266,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>50</v>
       </c>
@@ -1287,7 +1286,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>54</v>
       </c>
@@ -1307,7 +1306,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>58</v>
       </c>
@@ -1327,7 +1326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>62</v>
       </c>
@@ -1347,7 +1346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
@@ -1367,7 +1366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>71</v>
       </c>
@@ -1387,7 +1386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>75</v>
       </c>
@@ -1407,7 +1406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>79</v>
       </c>
@@ -1427,7 +1426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>82</v>
       </c>
@@ -1447,7 +1446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>86</v>
       </c>
@@ -1467,7 +1466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>89</v>
       </c>
@@ -1487,7 +1486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>93</v>
       </c>
@@ -1507,7 +1506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>96</v>
       </c>
@@ -1527,7 +1526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>100</v>
       </c>
@@ -1547,7 +1546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>104</v>
       </c>
@@ -1567,7 +1566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>109</v>
       </c>
@@ -1587,7 +1586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>113</v>
       </c>
@@ -1607,7 +1606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>117</v>
       </c>
@@ -1627,7 +1626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>120</v>
       </c>
@@ -1647,7 +1646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>124</v>
       </c>
@@ -1667,7 +1666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>128</v>
       </c>
@@ -1687,7 +1686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>133</v>
       </c>
@@ -1707,7 +1706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>138</v>
       </c>
@@ -1727,7 +1726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>143</v>
       </c>
@@ -1747,7 +1746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>147</v>
       </c>
@@ -1767,7 +1766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>152</v>
       </c>
@@ -1787,7 +1786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>157</v>
       </c>
@@ -1807,7 +1806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>161</v>
       </c>
@@ -1827,7 +1826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>166</v>
       </c>
@@ -1847,7 +1846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>170</v>
       </c>
@@ -1867,7 +1866,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>175</v>
       </c>
@@ -1887,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>179</v>
       </c>
@@ -1907,7 +1906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>184</v>
       </c>
@@ -1927,101 +1926,101 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="E45" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F45" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="B46" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="E45" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="F45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+      <c r="C46" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="E46" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="F46" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="B47" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="E46" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F46" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="E47" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="B48" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="E47" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="F47" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="D48" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="E48" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F48" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="B49" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="E48" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F48" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="D49" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="E49" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="F49" s="1">
         <v>1</v>

</xml_diff>

<commit_message>
#8 Fresh Altium BOM Genereated.
</commit_message>
<xml_diff>
--- a/Design-Files/BOM/Smart-Switch-v1.1.xlsx
+++ b/Design-Files/BOM/Smart-Switch-v1.1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\adamkop-smartswitch\Design-Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="3555" yWindow="3270" windowWidth="17280" windowHeight="8970"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="2370" windowHeight="105"/>
   </bookViews>
   <sheets>
     <sheet name="Smart-Switch-v1.1" sheetId="1" r:id="rId1"/>
@@ -22,23 +22,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="214">
   <si>
     <t>Comment</t>
   </si>
@@ -163,7 +152,7 @@
     <t>GRM188R61E106KA73D</t>
   </si>
   <si>
-    <t>0.1uf</t>
+    <t>0.1uF</t>
   </si>
   <si>
     <t>CAP CER 0.1UF 25V X5R 0201</t>
@@ -202,7 +191,7 @@
     <t>GRM033R61C105ME15D</t>
   </si>
   <si>
-    <t>22PF</t>
+    <t>22pF</t>
   </si>
   <si>
     <t>CAP CER 22PF 50V C0G/NP0 0201</t>
@@ -412,16 +401,16 @@
     <t>Test-point</t>
   </si>
   <si>
-    <t>DMN13H750S-7</t>
-  </si>
-  <si>
-    <t>MOSFET N-CH 130V 1A SOT23</t>
+    <t>MMBT3904M</t>
+  </si>
+  <si>
+    <t>40V 100mW 100@10mA,1V 200mA 300MHz 300mV@50mA,5mA NPN -55℃~+150℃@(Tj) SOT-723 Bipolar Transistors - BJT ROHS</t>
   </si>
   <si>
     <t>Q1</t>
   </si>
   <si>
-    <t>SOT-23</t>
+    <t>SOT-723</t>
   </si>
   <si>
     <t>10R</t>
@@ -433,7 +422,7 @@
     <t>R1</t>
   </si>
   <si>
-    <t>MO2WS VERTICAL TYPE</t>
+    <t>MO2WS Vertical Type</t>
   </si>
   <si>
     <t>Vertical Resistor</t>
@@ -502,7 +491,7 @@
     <t>RES SMD 10K OHM 1% 1/20W 0201</t>
   </si>
   <si>
-    <t>R7, R10, R14, R15</t>
+    <t>R7, R10, R15</t>
   </si>
   <si>
     <t>Res-0201</t>
@@ -538,9 +527,6 @@
     <t>RC0402FR-071KL</t>
   </si>
   <si>
-    <t>10k</t>
-  </si>
-  <si>
     <t>THERMISTOR NTC 10KOHM 3380K 0603</t>
   </si>
   <si>
@@ -550,19 +536,28 @@
     <t>B57332V5103F360</t>
   </si>
   <si>
-    <t>200K</t>
-  </si>
-  <si>
-    <t>750mW Thick Film Resistors ±5% ±200ppm/℃ 200kΩ 1210 Chip Resistor - Surface Mount ROHS</t>
+    <t>33K</t>
+  </si>
+  <si>
+    <t>RES SMD 33 KOHM 1% 1/2W 0805</t>
   </si>
   <si>
     <t>R12, R13</t>
   </si>
   <si>
-    <t>Res_1210</t>
-  </si>
-  <si>
-    <t>CR1210J30204G</t>
+    <t>ERJ-P06F3302V</t>
+  </si>
+  <si>
+    <t>4.7K</t>
+  </si>
+  <si>
+    <t>RES 4.7K OHM 1% 1/20W 0201</t>
+  </si>
+  <si>
+    <t>R14</t>
+  </si>
+  <si>
+    <t>RC0201FR-074K7L</t>
   </si>
   <si>
     <t>240R</t>
@@ -592,6 +587,18 @@
     <t>RCA0603100RFKEAHP</t>
   </si>
   <si>
+    <t>47K</t>
+  </si>
+  <si>
+    <t>RES 47K OHM 1% 1/20W 0201</t>
+  </si>
+  <si>
+    <t>R19</t>
+  </si>
+  <si>
+    <t>RC0201FR-0747KL</t>
+  </si>
+  <si>
     <t>B3U-1000P</t>
   </si>
   <si>
@@ -601,6 +608,12 @@
     <t>SW1, SW2</t>
   </si>
   <si>
+    <t>VIPER319XDTR</t>
+  </si>
+  <si>
+    <t>IC OFFLINE SWITCH MULT TOP 16SO</t>
+  </si>
+  <si>
     <t>U1</t>
   </si>
   <si>
@@ -656,12 +669,6 @@
   </si>
   <si>
     <t>X322540MPB4SI</t>
-  </si>
-  <si>
-    <t>VIPER319XDTR</t>
-  </si>
-  <si>
-    <t>IC OFFLINE SWITCH MULT TOP 16SO</t>
   </si>
 </sst>
 </file>
@@ -758,7 +765,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -770,7 +777,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -817,23 +824,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -869,23 +859,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1038,12 +1011,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="1" max="6" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1783,7 +1754,7 @@
         <v>156</v>
       </c>
       <c r="F37" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1828,19 +1799,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>136</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F40" s="1">
         <v>1</v>
@@ -1848,19 +1819,19 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>174</v>
       </c>
       <c r="F41" s="1">
         <v>2</v>
@@ -1868,19 +1839,19 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="F42" s="1">
         <v>1</v>
@@ -1888,39 +1859,39 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="D43" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>183</v>
-      </c>
       <c r="F43" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>184</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F44" s="1">
         <v>2</v>
@@ -1928,19 +1899,19 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>206</v>
+        <v>186</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>207</v>
+        <v>187</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>206</v>
+        <v>189</v>
       </c>
       <c r="F45" s="1">
         <v>1</v>
@@ -1948,22 +1919,22 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="E46" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F46" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2020,9 +1991,49 @@
         <v>204</v>
       </c>
       <c r="E49" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F49" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="F49" s="1">
+      <c r="B50" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="F50" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="F51" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>